<commit_message>
fix: se cambio el excel
</commit_message>
<xml_diff>
--- a/public/plantillas/censo.xlsx
+++ b/public/plantillas/censo.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpolo\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F92559C-58D8-4A7E-A068-728B5DD5B114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF4D957-2DA7-4C20-80AD-A10D4CB7C839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7F101705-DC27-4D52-9C41-1E983A9E60F3}"/>
   </bookViews>
   <sheets>
     <sheet name="C200" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="270">
   <si>
     <t>EDAD EN AÑOS CUMPLIDOS
 AL 31-03-2026</t>
@@ -175,12 +174,6 @@
     <t>{e_24_h}</t>
   </si>
   <si>
-    <t>{e_</t>
-  </si>
-  <si>
-    <t>_h}</t>
-  </si>
-  <si>
     <t>{e_16_h}</t>
   </si>
   <si>
@@ -203,9 +196,6 @@
   </si>
   <si>
     <t>{e_23_h}</t>
-  </si>
-  <si>
-    <t>_m}</t>
   </si>
   <si>
     <t>{e_16_m}</t>
@@ -4446,7 +4436,7 @@
         <v>28</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F12" s="11"/>
       <c r="G12" s="12"/>
@@ -4473,7 +4463,7 @@
         <v>29</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F13" s="11"/>
       <c r="G13" s="12"/>
@@ -4497,10 +4487,10 @@
       </c>
       <c r="C14" s="225"/>
       <c r="D14" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F14" s="11"/>
       <c r="G14" s="12"/>
@@ -4524,10 +4514,10 @@
       </c>
       <c r="C15" s="225"/>
       <c r="D15" s="10" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F15" s="11"/>
       <c r="G15" s="12"/>
@@ -4551,10 +4541,10 @@
       </c>
       <c r="C16" s="225"/>
       <c r="D16" s="10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F16" s="11"/>
       <c r="G16" s="12"/>
@@ -4578,10 +4568,10 @@
       </c>
       <c r="C17" s="225"/>
       <c r="D17" s="10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F17" s="11"/>
       <c r="G17" s="12"/>
@@ -4605,10 +4595,10 @@
       </c>
       <c r="C18" s="225"/>
       <c r="D18" s="10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F18" s="11"/>
       <c r="G18" s="12"/>
@@ -4632,10 +4622,10 @@
       </c>
       <c r="C19" s="225"/>
       <c r="D19" s="10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="12"/>
@@ -4659,10 +4649,10 @@
       </c>
       <c r="C20" s="225"/>
       <c r="D20" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F20" s="11"/>
       <c r="G20" s="12"/>
@@ -4686,10 +4676,10 @@
       </c>
       <c r="C21" s="225"/>
       <c r="D21" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F21" s="11"/>
       <c r="G21" s="12"/>
@@ -4716,7 +4706,7 @@
         <v>30</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F22" s="11"/>
       <c r="G22" s="12"/>
@@ -4740,10 +4730,10 @@
       </c>
       <c r="C23" s="225"/>
       <c r="D23" s="10" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F23" s="11"/>
       <c r="G23" s="12"/>
@@ -4767,10 +4757,10 @@
       </c>
       <c r="C24" s="225"/>
       <c r="D24" s="10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F24" s="11"/>
       <c r="G24" s="12"/>
@@ -4794,10 +4784,10 @@
       </c>
       <c r="C25" s="225"/>
       <c r="D25" s="10" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F25" s="11"/>
       <c r="G25" s="12"/>
@@ -4821,10 +4811,10 @@
       </c>
       <c r="C26" s="225"/>
       <c r="D26" s="10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F26" s="11"/>
       <c r="G26" s="12"/>
@@ -4848,10 +4838,10 @@
       </c>
       <c r="C27" s="225"/>
       <c r="D27" s="10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F27" s="11"/>
       <c r="G27" s="12"/>
@@ -4875,10 +4865,10 @@
       </c>
       <c r="C28" s="225"/>
       <c r="D28" s="10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F28" s="11"/>
       <c r="G28" s="12"/>
@@ -4902,10 +4892,10 @@
       </c>
       <c r="C29" s="225"/>
       <c r="D29" s="10" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F29" s="11"/>
       <c r="G29" s="12"/>
@@ -4929,10 +4919,10 @@
       </c>
       <c r="C30" s="227"/>
       <c r="D30" s="15" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F30" s="16"/>
       <c r="G30" s="17"/>
@@ -5169,10 +5159,10 @@
       <c r="E40" s="47"/>
       <c r="F40" s="48"/>
       <c r="G40" s="40" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H40" s="40" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I40" s="50"/>
       <c r="J40" s="51"/>
@@ -5199,10 +5189,10 @@
       <c r="E41" s="56"/>
       <c r="F41" s="57"/>
       <c r="G41" s="49" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="H41" s="49" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I41" s="11"/>
       <c r="J41" s="58"/>
@@ -5229,10 +5219,10 @@
       <c r="E42" s="56"/>
       <c r="F42" s="57"/>
       <c r="G42" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I42" s="11"/>
       <c r="J42" s="58"/>
@@ -5259,10 +5249,10 @@
       <c r="E43" s="56"/>
       <c r="F43" s="57"/>
       <c r="G43" s="10" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="I43" s="11"/>
       <c r="J43" s="58"/>
@@ -5289,10 +5279,10 @@
       <c r="E44" s="56"/>
       <c r="F44" s="57"/>
       <c r="G44" s="10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I44" s="11"/>
       <c r="J44" s="58"/>
@@ -5319,10 +5309,10 @@
       <c r="E45" s="56"/>
       <c r="F45" s="57"/>
       <c r="G45" s="10" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="I45" s="11"/>
       <c r="J45" s="58"/>
@@ -5349,10 +5339,10 @@
       <c r="E46" s="65"/>
       <c r="F46" s="66"/>
       <c r="G46" s="10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="67"/>
@@ -5401,7 +5391,7 @@
         <v>204</v>
       </c>
       <c r="C52" s="174" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D52" s="175"/>
       <c r="E52" s="175"/>
@@ -5434,14 +5424,14 @@
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="125"/>
       <c r="B54" s="176" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C54" s="177"/>
       <c r="D54" s="180" t="s">
         <v>1</v>
       </c>
       <c r="E54" s="126" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F54" s="127"/>
       <c r="G54" s="127"/>
@@ -5486,13 +5476,13 @@
         <v>2017</v>
       </c>
       <c r="N55" s="130" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="125"/>
       <c r="B56" s="131" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C56" s="132"/>
       <c r="D56" s="133">
@@ -5500,40 +5490,40 @@
         <v>0</v>
       </c>
       <c r="E56" s="134" t="s">
+        <v>243</v>
+      </c>
+      <c r="F56" s="135" t="s">
+        <v>244</v>
+      </c>
+      <c r="G56" s="135" t="s">
+        <v>245</v>
+      </c>
+      <c r="H56" s="135" t="s">
         <v>246</v>
       </c>
-      <c r="F56" s="135" t="s">
+      <c r="I56" s="135" t="s">
         <v>247</v>
       </c>
-      <c r="G56" s="135" t="s">
+      <c r="J56" s="135" t="s">
         <v>248</v>
       </c>
-      <c r="H56" s="135" t="s">
+      <c r="K56" s="135" t="s">
         <v>249</v>
       </c>
-      <c r="I56" s="135" t="s">
+      <c r="L56" s="135" t="s">
         <v>250</v>
       </c>
-      <c r="J56" s="135" t="s">
+      <c r="M56" s="135" t="s">
         <v>251</v>
       </c>
-      <c r="K56" s="135" t="s">
-        <v>252</v>
-      </c>
-      <c r="L56" s="135" t="s">
-        <v>253</v>
-      </c>
-      <c r="M56" s="135" t="s">
-        <v>254</v>
-      </c>
       <c r="N56" s="135" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="125"/>
       <c r="B57" s="63" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C57" s="65"/>
       <c r="D57" s="133">
@@ -5541,34 +5531,34 @@
         <v>0</v>
       </c>
       <c r="E57" s="134" t="s">
+        <v>252</v>
+      </c>
+      <c r="F57" s="135" t="s">
+        <v>253</v>
+      </c>
+      <c r="G57" s="135" t="s">
+        <v>254</v>
+      </c>
+      <c r="H57" s="135" t="s">
         <v>255</v>
       </c>
-      <c r="F57" s="135" t="s">
+      <c r="I57" s="135" t="s">
         <v>256</v>
       </c>
-      <c r="G57" s="135" t="s">
+      <c r="J57" s="135" t="s">
         <v>257</v>
       </c>
-      <c r="H57" s="135" t="s">
+      <c r="K57" s="135" t="s">
         <v>258</v>
       </c>
-      <c r="I57" s="135" t="s">
+      <c r="L57" s="135" t="s">
         <v>259</v>
       </c>
-      <c r="J57" s="135" t="s">
+      <c r="M57" s="135" t="s">
         <v>260</v>
       </c>
-      <c r="K57" s="135" t="s">
-        <v>261</v>
-      </c>
-      <c r="L57" s="135" t="s">
-        <v>262</v>
-      </c>
-      <c r="M57" s="135" t="s">
-        <v>263</v>
-      </c>
       <c r="N57" s="135" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="71" spans="1:25" ht="18" x14ac:dyDescent="0.25">
@@ -5577,7 +5567,7 @@
         <v>207</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D71" s="34"/>
       <c r="E71" s="35"/>
@@ -5632,10 +5622,10 @@
     <row r="73" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A73" s="69"/>
       <c r="B73" s="204" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C73" s="185" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D73" s="196"/>
       <c r="E73" s="196"/>
@@ -5652,10 +5642,10 @@
       <c r="L73" s="191"/>
       <c r="M73" s="69"/>
       <c r="N73" s="207" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="O73" s="185" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="P73" s="196"/>
       <c r="Q73" s="196"/>
@@ -5761,7 +5751,7 @@
     <row r="76" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="69"/>
       <c r="B76" s="72" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C76" s="73" t="s">
         <v>1</v>
@@ -5791,10 +5781,10 @@
       </c>
       <c r="M76" s="69"/>
       <c r="N76" s="76" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="O76" s="77" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="P76" s="78"/>
       <c r="Q76" s="78"/>
@@ -5814,19 +5804,19 @@
     <row r="77" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A77" s="69"/>
       <c r="B77" s="83" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C77" s="84" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D77" s="85"/>
       <c r="E77" s="85"/>
       <c r="F77" s="85"/>
       <c r="G77" s="86" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H77" s="86" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="I77" s="87"/>
       <c r="J77" s="88"/>
@@ -5834,10 +5824,10 @@
       <c r="L77" s="89"/>
       <c r="M77" s="69"/>
       <c r="N77" s="90" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O77" s="91" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="P77" s="56"/>
       <c r="Q77" s="56"/>
@@ -5857,7 +5847,7 @@
     <row r="78" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A78" s="69"/>
       <c r="B78" s="96" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C78" s="97"/>
       <c r="D78" s="97"/>
@@ -5871,10 +5861,10 @@
       <c r="L78" s="99"/>
       <c r="M78" s="69"/>
       <c r="N78" s="90" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="O78" s="91" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="P78" s="56"/>
       <c r="Q78" s="56"/>
@@ -5894,10 +5884,10 @@
     <row r="79" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A79" s="69"/>
       <c r="B79" s="100" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C79" s="101" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D79" s="47"/>
       <c r="E79" s="47"/>
@@ -5914,10 +5904,10 @@
       <c r="L79" s="105"/>
       <c r="M79" s="69"/>
       <c r="N79" s="90" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="O79" s="91" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="P79" s="56"/>
       <c r="Q79" s="56"/>
@@ -5937,19 +5927,19 @@
     <row r="80" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A80" s="69"/>
       <c r="B80" s="90" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C80" s="91" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D80" s="56"/>
       <c r="E80" s="56"/>
       <c r="F80" s="56"/>
       <c r="G80" s="92" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="H80" s="92" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="I80" s="93"/>
       <c r="J80" s="94"/>
@@ -5957,10 +5947,10 @@
       <c r="L80" s="95"/>
       <c r="M80" s="69"/>
       <c r="N80" s="90" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="O80" s="91" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="P80" s="56"/>
       <c r="Q80" s="56"/>
@@ -5980,10 +5970,10 @@
     <row r="81" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A81" s="69"/>
       <c r="B81" s="90" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C81" s="91" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D81" s="56"/>
       <c r="E81" s="56"/>
@@ -6000,10 +5990,10 @@
       <c r="L81" s="95"/>
       <c r="M81" s="69"/>
       <c r="N81" s="90" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="O81" s="91" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="P81" s="56"/>
       <c r="Q81" s="56"/>
@@ -6023,10 +6013,10 @@
     <row r="82" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A82" s="69"/>
       <c r="B82" s="90" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C82" s="91" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D82" s="56"/>
       <c r="E82" s="56"/>
@@ -6043,10 +6033,10 @@
       <c r="L82" s="95"/>
       <c r="M82" s="69"/>
       <c r="N82" s="90" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="O82" s="91" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="P82" s="56"/>
       <c r="Q82" s="56"/>
@@ -6066,19 +6056,19 @@
     <row r="83" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A83" s="69"/>
       <c r="B83" s="90" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C83" s="91" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D83" s="56"/>
       <c r="E83" s="56"/>
       <c r="F83" s="56"/>
       <c r="G83" s="92" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="H83" s="92" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I83" s="93"/>
       <c r="J83" s="94"/>
@@ -6086,10 +6076,10 @@
       <c r="L83" s="95"/>
       <c r="M83" s="69"/>
       <c r="N83" s="90" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="O83" s="106" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="P83" s="56"/>
       <c r="Q83" s="56"/>
@@ -6109,10 +6099,10 @@
     <row r="84" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A84" s="69"/>
       <c r="B84" s="90" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C84" s="91" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D84" s="56"/>
       <c r="E84" s="56"/>
@@ -6129,10 +6119,10 @@
       <c r="L84" s="95"/>
       <c r="M84" s="69"/>
       <c r="N84" s="90" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="O84" s="91" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="P84" s="56"/>
       <c r="Q84" s="56"/>
@@ -6152,10 +6142,10 @@
     <row r="85" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A85" s="69"/>
       <c r="B85" s="90" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C85" s="91" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D85" s="56"/>
       <c r="E85" s="56"/>
@@ -6172,10 +6162,10 @@
       <c r="L85" s="95"/>
       <c r="M85" s="69"/>
       <c r="N85" s="90" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="O85" s="91" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="P85" s="56"/>
       <c r="Q85" s="56"/>
@@ -6195,10 +6185,10 @@
     <row r="86" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A86" s="69"/>
       <c r="B86" s="90" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C86" s="91" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D86" s="56"/>
       <c r="E86" s="56"/>
@@ -6215,10 +6205,10 @@
       <c r="L86" s="95"/>
       <c r="M86" s="69"/>
       <c r="N86" s="90" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="O86" s="91" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="P86" s="56"/>
       <c r="Q86" s="56"/>
@@ -6238,10 +6228,10 @@
     <row r="87" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A87" s="69"/>
       <c r="B87" s="90" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C87" s="91" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D87" s="56"/>
       <c r="E87" s="56"/>
@@ -6258,10 +6248,10 @@
       <c r="L87" s="95"/>
       <c r="M87" s="69"/>
       <c r="N87" s="90" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="O87" s="91" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="P87" s="56"/>
       <c r="Q87" s="56"/>
@@ -6281,10 +6271,10 @@
     <row r="88" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A88" s="69"/>
       <c r="B88" s="90" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C88" s="91" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D88" s="56"/>
       <c r="E88" s="56"/>
@@ -6301,10 +6291,10 @@
       <c r="L88" s="95"/>
       <c r="M88" s="69"/>
       <c r="N88" s="90" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="O88" s="91" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="P88" s="56"/>
       <c r="Q88" s="56"/>
@@ -6324,10 +6314,10 @@
     <row r="89" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A89" s="69"/>
       <c r="B89" s="90" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C89" s="91" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D89" s="56"/>
       <c r="E89" s="56"/>
@@ -6344,10 +6334,10 @@
       <c r="L89" s="95"/>
       <c r="M89" s="69"/>
       <c r="N89" s="90" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="O89" s="91" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="P89" s="56"/>
       <c r="Q89" s="56"/>
@@ -6367,10 +6357,10 @@
     <row r="90" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A90" s="69"/>
       <c r="B90" s="90" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C90" s="91" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D90" s="56"/>
       <c r="E90" s="56"/>
@@ -6387,10 +6377,10 @@
       <c r="L90" s="95"/>
       <c r="M90" s="69"/>
       <c r="N90" s="90" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="O90" s="91" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="P90" s="56"/>
       <c r="Q90" s="56"/>
@@ -6410,10 +6400,10 @@
     <row r="91" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A91" s="69"/>
       <c r="B91" s="90" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C91" s="91" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D91" s="56"/>
       <c r="E91" s="56"/>
@@ -6430,10 +6420,10 @@
       <c r="L91" s="95"/>
       <c r="M91" s="69"/>
       <c r="N91" s="90" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="O91" s="91" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="P91" s="56"/>
       <c r="Q91" s="56"/>
@@ -6453,10 +6443,10 @@
     <row r="92" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A92" s="69"/>
       <c r="B92" s="90" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C92" s="91" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D92" s="56"/>
       <c r="E92" s="56"/>
@@ -6473,10 +6463,10 @@
       <c r="L92" s="95"/>
       <c r="M92" s="69"/>
       <c r="N92" s="90" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="O92" s="91" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="P92" s="56"/>
       <c r="Q92" s="56"/>
@@ -6496,10 +6486,10 @@
     <row r="93" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A93" s="69"/>
       <c r="B93" s="90" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C93" s="91" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D93" s="56"/>
       <c r="E93" s="56"/>
@@ -6516,10 +6506,10 @@
       <c r="L93" s="95"/>
       <c r="M93" s="69"/>
       <c r="N93" s="90" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="O93" s="91" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="P93" s="56"/>
       <c r="Q93" s="56"/>
@@ -6539,10 +6529,10 @@
     <row r="94" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A94" s="69"/>
       <c r="B94" s="90" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C94" s="91" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D94" s="56"/>
       <c r="E94" s="56"/>
@@ -6559,10 +6549,10 @@
       <c r="L94" s="95"/>
       <c r="M94" s="69"/>
       <c r="N94" s="90" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="O94" s="91" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="P94" s="56"/>
       <c r="Q94" s="56"/>
@@ -6582,10 +6572,10 @@
     <row r="95" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A95" s="69"/>
       <c r="B95" s="90" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C95" s="91" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D95" s="56"/>
       <c r="E95" s="56"/>
@@ -6602,10 +6592,10 @@
       <c r="L95" s="95"/>
       <c r="M95" s="69"/>
       <c r="N95" s="90" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="O95" s="91" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="P95" s="56"/>
       <c r="Q95" s="56"/>
@@ -6625,10 +6615,10 @@
     <row r="96" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A96" s="69"/>
       <c r="B96" s="90" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C96" s="91" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D96" s="56"/>
       <c r="E96" s="56"/>
@@ -6645,10 +6635,10 @@
       <c r="L96" s="95"/>
       <c r="M96" s="69"/>
       <c r="N96" s="90" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="O96" s="91" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="P96" s="56"/>
       <c r="Q96" s="56"/>
@@ -6668,10 +6658,10 @@
     <row r="97" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A97" s="69"/>
       <c r="B97" s="90" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C97" s="91" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D97" s="56"/>
       <c r="E97" s="56"/>
@@ -6688,10 +6678,10 @@
       <c r="L97" s="95"/>
       <c r="M97" s="69"/>
       <c r="N97" s="90" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="O97" s="91" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="P97" s="56"/>
       <c r="Q97" s="56"/>
@@ -6711,10 +6701,10 @@
     <row r="98" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A98" s="69"/>
       <c r="B98" s="90" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C98" s="91" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D98" s="56"/>
       <c r="E98" s="56"/>
@@ -6731,10 +6721,10 @@
       <c r="L98" s="95"/>
       <c r="M98" s="69"/>
       <c r="N98" s="90" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="O98" s="91" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="P98" s="56"/>
       <c r="Q98" s="56"/>
@@ -6754,10 +6744,10 @@
     <row r="99" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A99" s="69"/>
       <c r="B99" s="90" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C99" s="91" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D99" s="56"/>
       <c r="E99" s="56"/>
@@ -6774,10 +6764,10 @@
       <c r="L99" s="95"/>
       <c r="M99" s="69"/>
       <c r="N99" s="90" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="O99" s="91" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="P99" s="56"/>
       <c r="Q99" s="56"/>
@@ -6797,10 +6787,10 @@
     <row r="100" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A100" s="69"/>
       <c r="B100" s="90" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C100" s="91" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D100" s="56"/>
       <c r="E100" s="56"/>
@@ -6817,10 +6807,10 @@
       <c r="L100" s="95"/>
       <c r="M100" s="69"/>
       <c r="N100" s="90" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="O100" s="91" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="P100" s="56"/>
       <c r="Q100" s="56"/>
@@ -6840,10 +6830,10 @@
     <row r="101" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A101" s="69"/>
       <c r="B101" s="90" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C101" s="91" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D101" s="56"/>
       <c r="E101" s="56"/>
@@ -6860,20 +6850,20 @@
       <c r="L101" s="95"/>
       <c r="M101" s="69"/>
       <c r="N101" s="90" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="O101" s="91" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="P101" s="56"/>
       <c r="Q101" s="56"/>
       <c r="R101" s="56"/>
       <c r="S101" s="56"/>
       <c r="T101" s="92" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="U101" s="92" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="V101" s="93"/>
       <c r="W101" s="94"/>
@@ -6883,10 +6873,10 @@
     <row r="102" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A102" s="69"/>
       <c r="B102" s="90" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C102" s="91" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D102" s="56"/>
       <c r="E102" s="56"/>
@@ -6903,7 +6893,7 @@
       <c r="L102" s="95"/>
       <c r="M102" s="69"/>
       <c r="N102" s="96" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="O102" s="97"/>
       <c r="P102" s="97"/>
@@ -6920,10 +6910,10 @@
     <row r="103" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A103" s="69"/>
       <c r="B103" s="90" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C103" s="91" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D103" s="56"/>
       <c r="E103" s="56"/>
@@ -6940,10 +6930,10 @@
       <c r="L103" s="95"/>
       <c r="M103" s="69"/>
       <c r="N103" s="100" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="O103" s="101" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="P103" s="47"/>
       <c r="Q103" s="47"/>
@@ -6963,10 +6953,10 @@
     <row r="104" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A104" s="69"/>
       <c r="B104" s="90" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C104" s="91" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D104" s="56"/>
       <c r="E104" s="56"/>
@@ -6983,10 +6973,10 @@
       <c r="L104" s="95"/>
       <c r="M104" s="69"/>
       <c r="N104" s="90" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="O104" s="91" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="P104" s="56"/>
       <c r="Q104" s="56"/>
@@ -7006,10 +6996,10 @@
     <row r="105" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A105" s="69"/>
       <c r="B105" s="90" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C105" s="91" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D105" s="56"/>
       <c r="E105" s="56"/>
@@ -7026,10 +7016,10 @@
       <c r="L105" s="95"/>
       <c r="M105" s="69"/>
       <c r="N105" s="90" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="O105" s="91" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="P105" s="56"/>
       <c r="Q105" s="56"/>
@@ -7049,10 +7039,10 @@
     <row r="106" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A106" s="69"/>
       <c r="B106" s="90" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C106" s="91" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D106" s="56"/>
       <c r="E106" s="56"/>
@@ -7069,10 +7059,10 @@
       <c r="L106" s="95"/>
       <c r="M106" s="69"/>
       <c r="N106" s="90" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="O106" s="91" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="P106" s="56"/>
       <c r="Q106" s="56"/>
@@ -7092,10 +7082,10 @@
     <row r="107" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A107" s="69"/>
       <c r="B107" s="90" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C107" s="91" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D107" s="56"/>
       <c r="E107" s="56"/>
@@ -7112,10 +7102,10 @@
       <c r="L107" s="95"/>
       <c r="M107" s="69"/>
       <c r="N107" s="90" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="O107" s="91" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="P107" s="56"/>
       <c r="Q107" s="56"/>
@@ -7135,10 +7125,10 @@
     <row r="108" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A108" s="69"/>
       <c r="B108" s="90" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C108" s="91" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D108" s="56"/>
       <c r="E108" s="56"/>
@@ -7155,10 +7145,10 @@
       <c r="L108" s="95"/>
       <c r="M108" s="69"/>
       <c r="N108" s="90" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="O108" s="91" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="P108" s="56"/>
       <c r="Q108" s="56"/>
@@ -7178,10 +7168,10 @@
     <row r="109" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A109" s="69"/>
       <c r="B109" s="90" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C109" s="91" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D109" s="56"/>
       <c r="E109" s="56"/>
@@ -7198,10 +7188,10 @@
       <c r="L109" s="95"/>
       <c r="M109" s="69"/>
       <c r="N109" s="90" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="O109" s="91" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="P109" s="56"/>
       <c r="Q109" s="56"/>
@@ -7221,10 +7211,10 @@
     <row r="110" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A110" s="69"/>
       <c r="B110" s="108" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C110" s="109" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D110" s="65"/>
       <c r="E110" s="65"/>
@@ -7241,20 +7231,20 @@
       <c r="L110" s="113"/>
       <c r="M110" s="114"/>
       <c r="N110" s="115" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="O110" s="116" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="P110" s="65"/>
       <c r="Q110" s="65"/>
       <c r="R110" s="65"/>
       <c r="S110" s="65"/>
       <c r="T110" s="117" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="U110" s="117" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="V110" s="118"/>
       <c r="W110" s="119"/>
@@ -7264,7 +7254,7 @@
     <row r="111" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A111" s="69"/>
       <c r="B111" s="1" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C111" s="121"/>
       <c r="D111" s="121"/>
@@ -7292,29 +7282,29 @@
     </row>
     <row r="113" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C113" s="182" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D113" s="183"/>
       <c r="E113" s="183"/>
       <c r="F113" s="184"/>
       <c r="G113" s="92" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H113" s="92" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="O113" s="122" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="P113" s="123"/>
       <c r="Q113" s="123"/>
       <c r="R113" s="123"/>
       <c r="S113" s="123"/>
       <c r="T113" s="124" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="U113" s="124" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="116" spans="1:21" ht="18" x14ac:dyDescent="0.25">
@@ -7323,7 +7313,7 @@
         <v>208</v>
       </c>
       <c r="C116" s="21" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D116" s="34"/>
       <c r="E116" s="35"/>
@@ -7350,12 +7340,12 @@
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="1"/>
       <c r="B118" s="158" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C118" s="159"/>
       <c r="D118" s="160"/>
       <c r="E118" s="164" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="F118" s="165"/>
       <c r="G118" s="168" t="s">
@@ -7409,7 +7399,7 @@
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="1"/>
       <c r="B121" s="139" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C121" s="140"/>
       <c r="D121" s="141"/>
@@ -7419,7 +7409,7 @@
       </c>
       <c r="F121" s="146"/>
       <c r="G121" s="147" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="H121" s="148"/>
       <c r="I121" s="149"/>
@@ -7429,7 +7419,7 @@
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="1"/>
       <c r="B122" s="139" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C122" s="140"/>
       <c r="D122" s="141"/>
@@ -7439,7 +7429,7 @@
       </c>
       <c r="F122" s="146"/>
       <c r="G122" s="147" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="H122" s="148"/>
       <c r="I122" s="149"/>
@@ -7449,7 +7439,7 @@
     <row r="123" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="1"/>
       <c r="B123" s="142" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C123" s="143"/>
       <c r="D123" s="144"/>
@@ -7459,7 +7449,7 @@
       </c>
       <c r="F123" s="146"/>
       <c r="G123" s="151" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="H123" s="152"/>
       <c r="I123" s="153"/>
@@ -7562,297 +7552,4 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16A570E0-EEA4-47A0-BB88-2EF3C853EFF7}">
-  <dimension ref="B4:O13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4">
-        <v>15</v>
-      </c>
-      <c r="G4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" t="str">
-        <f>_xlfn.CONCAT(E4:G4)</f>
-        <v>{e_15_h}</v>
-      </c>
-      <c r="L4" t="s">
-        <v>31</v>
-      </c>
-      <c r="M4">
-        <v>15</v>
-      </c>
-      <c r="N4" t="s">
-        <v>41</v>
-      </c>
-      <c r="O4" t="str">
-        <f>_xlfn.CONCAT(L4:N4)</f>
-        <v>{e_15_m}</v>
-      </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5">
-        <v>16</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" t="str">
-        <f t="shared" ref="H5:H13" si="0">_xlfn.CONCAT(E5:G5)</f>
-        <v>{e_16_h}</v>
-      </c>
-      <c r="L5" t="s">
-        <v>31</v>
-      </c>
-      <c r="M5">
-        <v>16</v>
-      </c>
-      <c r="N5" t="s">
-        <v>41</v>
-      </c>
-      <c r="O5" t="str">
-        <f>_xlfn.CONCAT(L5:N5)</f>
-        <v>{e_16_m}</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6">
-        <v>17</v>
-      </c>
-      <c r="G6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" t="str">
-        <f t="shared" si="0"/>
-        <v>{e_17_h}</v>
-      </c>
-      <c r="L6" t="s">
-        <v>31</v>
-      </c>
-      <c r="M6">
-        <v>17</v>
-      </c>
-      <c r="N6" t="s">
-        <v>41</v>
-      </c>
-      <c r="O6" t="str">
-        <f t="shared" ref="O6:O13" si="1">_xlfn.CONCAT(L6:N6)</f>
-        <v>{e_17_m}</v>
-      </c>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7">
-        <v>18</v>
-      </c>
-      <c r="G7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H7" t="str">
-        <f t="shared" si="0"/>
-        <v>{e_18_h}</v>
-      </c>
-      <c r="L7" t="s">
-        <v>31</v>
-      </c>
-      <c r="M7">
-        <v>18</v>
-      </c>
-      <c r="N7" t="s">
-        <v>41</v>
-      </c>
-      <c r="O7" t="str">
-        <f t="shared" si="1"/>
-        <v>{e_18_m}</v>
-      </c>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8">
-        <v>19</v>
-      </c>
-      <c r="G8" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" t="str">
-        <f t="shared" si="0"/>
-        <v>{e_19_h}</v>
-      </c>
-      <c r="L8" t="s">
-        <v>31</v>
-      </c>
-      <c r="M8">
-        <v>19</v>
-      </c>
-      <c r="N8" t="s">
-        <v>41</v>
-      </c>
-      <c r="O8" t="str">
-        <f t="shared" si="1"/>
-        <v>{e_19_m}</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9">
-        <v>20</v>
-      </c>
-      <c r="G9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" t="str">
-        <f t="shared" si="0"/>
-        <v>{e_20_h}</v>
-      </c>
-      <c r="L9" t="s">
-        <v>31</v>
-      </c>
-      <c r="M9">
-        <v>20</v>
-      </c>
-      <c r="N9" t="s">
-        <v>41</v>
-      </c>
-      <c r="O9" t="str">
-        <f t="shared" si="1"/>
-        <v>{e_20_m}</v>
-      </c>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F10">
-        <v>21</v>
-      </c>
-      <c r="G10" t="s">
-        <v>32</v>
-      </c>
-      <c r="H10" t="str">
-        <f t="shared" si="0"/>
-        <v>{e_21_h}</v>
-      </c>
-      <c r="L10" t="s">
-        <v>31</v>
-      </c>
-      <c r="M10">
-        <v>21</v>
-      </c>
-      <c r="N10" t="s">
-        <v>41</v>
-      </c>
-      <c r="O10" t="str">
-        <f t="shared" si="1"/>
-        <v>{e_21_m}</v>
-      </c>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E11" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11">
-        <v>22</v>
-      </c>
-      <c r="G11" t="s">
-        <v>32</v>
-      </c>
-      <c r="H11" t="str">
-        <f t="shared" si="0"/>
-        <v>{e_22_h}</v>
-      </c>
-      <c r="L11" t="s">
-        <v>31</v>
-      </c>
-      <c r="M11">
-        <v>22</v>
-      </c>
-      <c r="N11" t="s">
-        <v>41</v>
-      </c>
-      <c r="O11" t="str">
-        <f t="shared" si="1"/>
-        <v>{e_22_m}</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E12" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12">
-        <v>23</v>
-      </c>
-      <c r="G12" t="s">
-        <v>32</v>
-      </c>
-      <c r="H12" t="str">
-        <f t="shared" si="0"/>
-        <v>{e_23_h}</v>
-      </c>
-      <c r="L12" t="s">
-        <v>31</v>
-      </c>
-      <c r="M12">
-        <v>23</v>
-      </c>
-      <c r="N12" t="s">
-        <v>41</v>
-      </c>
-      <c r="O12" t="str">
-        <f t="shared" si="1"/>
-        <v>{e_23_m}</v>
-      </c>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F13">
-        <v>24</v>
-      </c>
-      <c r="G13" t="s">
-        <v>32</v>
-      </c>
-      <c r="H13" t="str">
-        <f t="shared" si="0"/>
-        <v>{e_24_h}</v>
-      </c>
-      <c r="L13" t="s">
-        <v>31</v>
-      </c>
-      <c r="M13">
-        <v>24</v>
-      </c>
-      <c r="N13" t="s">
-        <v>41</v>
-      </c>
-      <c r="O13" t="str">
-        <f t="shared" si="1"/>
-        <v>{e_24_m}</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>